<commit_message>
Fix item-to-price mapping, unify xlsx layout (row heights, headers, print fit), update final top with market costs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JQLkwre52iMXL7eAYSL71v
</commit_message>
<xml_diff>
--- a/CLOTHES_FACTORY_PRICES_1410.xlsx
+++ b/CLOTHES_FACTORY_PRICES_1410.xlsx
@@ -71,32 +71,41 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -460,7 +469,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -472,7 +481,7 @@
     <col width="80" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="18" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>0358200022926000030 — Ростов, обмундирование спасателей (44-ФЗ аукцион, 19.10)</t>
@@ -483,7 +492,7 @@
       <c r="D1" s="2" t="n"/>
       <c r="E1" s="2" t="n"/>
     </row>
-    <row r="2">
+    <row r="2" ht="48" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Позиция</t>
@@ -510,8 +519,8 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="3" ht="32" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>Костюм спасателя зимний</t>
         </is>
@@ -519,20 +528,20 @@
       <c r="B3" s="2" t="n">
         <v>168</v>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="C3" s="5" t="n">
         <v>5000</v>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="D3" s="5" t="n">
         <v>840000</v>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>правило клиента; рынок опт 3 549–5 810 (Иваново), розн. МЧС 14 461</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Костюм спасателя летний</t>
         </is>
@@ -540,20 +549,20 @@
       <c r="B4" s="2" t="n">
         <v>241</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="C4" s="5" t="n">
         <v>3500</v>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="D4" s="5" t="n">
         <v>843500</v>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>правило клиента; рынок МЧС 2 490–5 995</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Комбинезон спасателя зимний</t>
         </is>
@@ -561,20 +570,20 @@
       <c r="B5" s="2" t="n">
         <v>208</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="5" t="n">
         <v>7100</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="5" t="n">
         <v>1476800</v>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Спецобъединение ПИЛОТ 10 199 −30% опт [оценка]; клиентский 5 000 — оптимистично</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Комбинезон спасателя летний</t>
         </is>
@@ -582,20 +591,20 @@
       <c r="B6" s="2" t="n">
         <v>239</v>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C6" s="5" t="n">
         <v>3766</v>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D6" s="5" t="n">
         <v>900074</v>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>ivuniforma Р-11-87 опт 3 766</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="7" ht="32" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Футболка форменная (с нанесением)</t>
         </is>
@@ -603,122 +612,122 @@
       <c r="B7" s="2" t="n">
         <v>268</v>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="C7" s="5" t="n">
         <v>350</v>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="D7" s="5" t="n">
         <v>93800</v>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>Иваново опт 211–270 + нанесение ~100 [оценка]</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+    <row r="8" ht="32" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Закупка итого</t>
         </is>
       </c>
       <c r="B8" s="2" t="n"/>
       <c r="C8" s="2" t="n"/>
-      <c r="D8" s="6" t="n">
+      <c r="D8" s="7" t="n">
         <v>4154174</v>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>Пересчёт с реальными ценами комбинезонов (раньше приравнивали к комплектам)</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+    <row r="9" ht="32" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Доставка</t>
         </is>
       </c>
       <c r="B9" s="2" t="n"/>
       <c r="C9" s="2" t="n"/>
-      <c r="D9" s="6" t="n">
+      <c r="D9" s="7" t="n">
         <v>111495</v>
       </c>
       <c r="E9" s="2" t="n"/>
     </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>НМЦК</t>
         </is>
       </c>
       <c r="B10" s="2" t="n"/>
       <c r="C10" s="2" t="n"/>
-      <c r="D10" s="6" t="n">
+      <c r="D10" s="7" t="n">
         <v>6224420.7</v>
       </c>
       <c r="E10" s="2" t="n"/>
     </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>Маржа при НМЦК</t>
         </is>
       </c>
       <c r="B11" s="2" t="n"/>
       <c r="C11" s="2" t="n"/>
-      <c r="D11" s="7" t="n">
+      <c r="D11" s="8" t="n">
         <v>0.314688192589553</v>
       </c>
       <c r="E11" s="2" t="n"/>
     </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+    <row r="12" ht="32" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>Чистая прибыль при НМЦК</t>
         </is>
       </c>
       <c r="B12" s="2" t="n"/>
       <c r="C12" s="2" t="n"/>
-      <c r="D12" s="6" t="n">
+      <c r="D12" s="7" t="n">
         <v>1503407.887527672</v>
       </c>
       <c r="E12" s="2" t="n"/>
     </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>Чистая прибыль при снижении 17%</t>
         </is>
       </c>
       <c r="B13" s="2" t="n"/>
       <c r="C13" s="2" t="n"/>
-      <c r="D13" s="6" t="n">
+      <c r="D13" s="7" t="n">
         <v>611174.5267068711</v>
       </c>
       <c r="E13" s="2" t="n"/>
     </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+    <row r="14" ht="32" customHeight="1">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>Безубыток до снижения</t>
         </is>
       </c>
       <c r="B14" s="2" t="n"/>
       <c r="C14" s="2" t="n"/>
-      <c r="D14" s="7" t="n">
+      <c r="D14" s="8" t="n">
         <v>0.2864489853244075</v>
       </c>
       <c r="E14" s="2" t="n"/>
     </row>
-    <row r="15">
+    <row r="15" ht="32" customHeight="1">
       <c r="A15" s="2" t="n"/>
       <c r="B15" s="2" t="n"/>
       <c r="C15" s="2" t="n"/>
       <c r="D15" s="2" t="n"/>
       <c r="E15" s="2" t="n"/>
     </row>
-    <row r="16">
-      <c r="A16" s="1" t="inlineStr">
+    <row r="16" ht="32" customHeight="1">
+      <c r="A16" s="9" t="inlineStr">
         <is>
           <t>32616443256 — Якутия ГПС, форменная одежда (223-ФЗ, 15.10)</t>
         </is>
@@ -728,35 +737,35 @@
       <c r="D16" s="2" t="n"/>
       <c r="E16" s="2" t="n"/>
     </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+    <row r="17" ht="32" customHeight="1">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>Позиция</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" s="10" t="inlineStr">
         <is>
           <t>Кол-во</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C17" s="10" t="inlineStr">
         <is>
           <t>Цена закупки, ₽</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D17" s="10" t="inlineStr">
         <is>
           <t>Сумма, ₽</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E17" s="10" t="inlineStr">
         <is>
           <t>Откуда цена</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="18" ht="32" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Костюм летний полевой</t>
         </is>
@@ -764,20 +773,20 @@
       <c r="B18" s="2" t="n">
         <v>405</v>
       </c>
-      <c r="C18" s="4" t="n">
+      <c r="C18" s="5" t="n">
         <v>3500</v>
       </c>
-      <c r="D18" s="4" t="n">
+      <c r="D18" s="5" t="n">
         <v>1417500</v>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>правило клиента; рынок опт 1 600–2 490 (Ивсотекс), розн. 4 600+ (Сплав)</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+    <row r="19" ht="32" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Зимняя форменная одежда (IV пояс)</t>
         </is>
@@ -785,122 +794,122 @@
       <c r="B19" s="2" t="n">
         <v>150</v>
       </c>
-      <c r="C19" s="4" t="n">
+      <c r="C19" s="5" t="n">
         <v>8543</v>
       </c>
-      <c r="D19" s="4" t="n">
+      <c r="D19" s="5" t="n">
         <v>1281450</v>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>Спецстандарт «Север» (тройка) 8 543; СпецТекс №265 IV пояс 4 600; Надым 9 760</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
+    <row r="20" ht="32" customHeight="1">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>Закупка итого</t>
         </is>
       </c>
       <c r="B20" s="2" t="n"/>
       <c r="C20" s="2" t="n"/>
-      <c r="D20" s="6" t="n">
+      <c r="D20" s="7" t="n">
         <v>2698950</v>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t>Зимняя — по костюму IV пояса; если «особый пояс −45» уровня Северный шельф 24 000 — убыток</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
+    <row r="21" ht="32" customHeight="1">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>Доставка</t>
         </is>
       </c>
       <c r="B21" s="2" t="n"/>
       <c r="C21" s="2" t="n"/>
-      <c r="D21" s="6" t="n">
+      <c r="D21" s="7" t="n">
         <v>150000</v>
       </c>
       <c r="E21" s="2" t="n"/>
     </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
+    <row r="22" ht="32" customHeight="1">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>НМЦК</t>
         </is>
       </c>
       <c r="B22" s="2" t="n"/>
       <c r="C22" s="2" t="n"/>
-      <c r="D22" s="6" t="n">
+      <c r="D22" s="7" t="n">
         <v>4999001.85</v>
       </c>
       <c r="E22" s="2" t="n"/>
     </row>
-    <row r="23">
-      <c r="A23" s="5" t="inlineStr">
+    <row r="23" ht="32" customHeight="1">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>Маржа при НМЦК</t>
         </is>
       </c>
       <c r="B23" s="2" t="n"/>
       <c r="C23" s="2" t="n"/>
-      <c r="D23" s="7" t="n">
+      <c r="D23" s="8" t="n">
         <v>0.4300962301104169</v>
       </c>
       <c r="E23" s="2" t="n"/>
     </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr">
+    <row r="24" ht="32" customHeight="1">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>Чистая прибыль при НМЦК</t>
         </is>
       </c>
       <c r="B24" s="2" t="n"/>
       <c r="C24" s="2" t="n"/>
-      <c r="D24" s="6" t="n">
+      <c r="D24" s="7" t="n">
         <v>1713936.366769315</v>
       </c>
       <c r="E24" s="2" t="n"/>
     </row>
-    <row r="25">
-      <c r="A25" s="5" t="inlineStr">
+    <row r="25" ht="32" customHeight="1">
+      <c r="A25" s="6" t="inlineStr">
         <is>
           <t>Чистая прибыль при снижении 15%</t>
         </is>
       </c>
       <c r="B25" s="2" t="n"/>
       <c r="C25" s="2" t="n"/>
-      <c r="D25" s="6" t="n">
+      <c r="D25" s="7" t="n">
         <v>1081662.612781315</v>
       </c>
       <c r="E25" s="2" t="n"/>
     </row>
-    <row r="26">
-      <c r="A26" s="5" t="inlineStr">
+    <row r="26" ht="32" customHeight="1">
+      <c r="A26" s="6" t="inlineStr">
         <is>
           <t>Безубыток до снижения</t>
         </is>
       </c>
       <c r="B26" s="2" t="n"/>
       <c r="C26" s="2" t="n"/>
-      <c r="D26" s="7" t="n">
+      <c r="D26" s="8" t="n">
         <v>0.4066125683595537</v>
       </c>
       <c r="E26" s="2" t="n"/>
     </row>
-    <row r="27">
+    <row r="27" ht="32" customHeight="1">
       <c r="A27" s="2" t="n"/>
       <c r="B27" s="2" t="n"/>
       <c r="C27" s="2" t="n"/>
       <c r="D27" s="2" t="n"/>
       <c r="E27" s="2" t="n"/>
     </row>
-    <row r="28">
-      <c r="A28" s="1" t="inlineStr">
+    <row r="28" ht="32" customHeight="1">
+      <c r="A28" s="9" t="inlineStr">
         <is>
           <t>32616431081 — ФБУ, спецодежда 18 позиций (223-ФЗ, 19.10)</t>
         </is>
@@ -910,35 +919,35 @@
       <c r="D28" s="2" t="n"/>
       <c r="E28" s="2" t="n"/>
     </row>
-    <row r="29">
-      <c r="A29" s="3" t="inlineStr">
+    <row r="29" ht="32" customHeight="1">
+      <c r="A29" s="10" t="inlineStr">
         <is>
           <t>Позиция</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B29" s="10" t="inlineStr">
         <is>
           <t>Кол-во</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr">
+      <c r="C29" s="10" t="inlineStr">
         <is>
           <t>Цена закупки, ₽</t>
         </is>
       </c>
-      <c r="D29" s="3" t="inlineStr">
+      <c r="D29" s="10" t="inlineStr">
         <is>
           <t>Сумма, ₽</t>
         </is>
       </c>
-      <c r="E29" s="3" t="inlineStr">
+      <c r="E29" s="10" t="inlineStr">
         <is>
           <t>Откуда цена</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+    <row r="30" ht="32" customHeight="1">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>Жилет сигнальный</t>
         </is>
@@ -946,20 +955,20 @@
       <c r="B30" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="C30" s="4" t="n">
+      <c r="C30" s="5" t="n">
         <v>320</v>
       </c>
-      <c r="D30" s="4" t="n">
+      <c r="D30" s="5" t="n">
         <v>4480</v>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="E30" s="4" t="inlineStr">
         <is>
           <t>Фабрикант 260–320</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+    <row r="31" ht="32" customHeight="1">
+      <c r="A31" s="4" t="inlineStr">
         <is>
           <t>Жилет утепленный</t>
         </is>
@@ -967,20 +976,20 @@
       <c r="B31" s="2" t="n">
         <v>64</v>
       </c>
-      <c r="C31" s="4" t="n">
+      <c r="C31" s="5" t="n">
         <v>1190</v>
       </c>
-      <c r="D31" s="4" t="n">
+      <c r="D31" s="5" t="n">
         <v>76160</v>
       </c>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="E31" s="4" t="inlineStr">
         <is>
           <t>ivuniforma опт 1 190</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+    <row r="32" ht="32" customHeight="1">
+      <c r="A32" s="4" t="inlineStr">
         <is>
           <t>Костюм противоэнцефалитный</t>
         </is>
@@ -988,20 +997,20 @@
       <c r="B32" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C32" s="4" t="n">
+      <c r="C32" s="5" t="n">
         <v>975</v>
       </c>
-      <c r="D32" s="4" t="n">
+      <c r="D32" s="5" t="n">
         <v>975</v>
       </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="E32" s="4" t="inlineStr">
         <is>
           <t>Фабрикант 975 / Ивсотекс 1 250</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+    <row r="33" ht="32" customHeight="1">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>Костюм летний от мех. воздействий (муж+жен)</t>
         </is>
@@ -1009,20 +1018,20 @@
       <c r="B33" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="C33" s="4" t="n">
+      <c r="C33" s="5" t="n">
         <v>1715</v>
       </c>
-      <c r="D33" s="4" t="n">
+      <c r="D33" s="5" t="n">
         <v>41160</v>
       </c>
-      <c r="E33" s="2" t="inlineStr">
+      <c r="E33" s="4" t="inlineStr">
         <is>
           <t>ivuniforma опт 1 610–1 715</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+    <row r="34" ht="32" customHeight="1">
+      <c r="A34" s="4" t="inlineStr">
         <is>
           <t>Куртка зимняя</t>
         </is>
@@ -1030,20 +1039,20 @@
       <c r="B34" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="C34" s="4" t="n">
+      <c r="C34" s="5" t="n">
         <v>2688</v>
       </c>
-      <c r="D34" s="4" t="n">
+      <c r="D34" s="5" t="n">
         <v>53760</v>
       </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="E34" s="4" t="inlineStr">
         <is>
           <t>ivuniforma опт 2 688</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+    <row r="35" ht="32" customHeight="1">
+      <c r="A35" s="4" t="inlineStr">
         <is>
           <t>Полукомбинезон зимний</t>
         </is>
@@ -1051,20 +1060,20 @@
       <c r="B35" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="C35" s="4" t="n">
+      <c r="C35" s="5" t="n">
         <v>958</v>
       </c>
-      <c r="D35" s="4" t="n">
+      <c r="D35" s="5" t="n">
         <v>19160</v>
       </c>
-      <c r="E35" s="2" t="inlineStr">
+      <c r="E35" s="4" t="inlineStr">
         <is>
           <t>Спецстандарт 958</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+    <row r="36" ht="32" customHeight="1">
+      <c r="A36" s="4" t="inlineStr">
         <is>
           <t>Костюм сигнальный летний</t>
         </is>
@@ -1072,20 +1081,20 @@
       <c r="B36" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C36" s="4" t="n">
+      <c r="C36" s="5" t="n">
         <v>6112</v>
       </c>
-      <c r="D36" s="4" t="n">
+      <c r="D36" s="5" t="n">
         <v>24448</v>
       </c>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="E36" s="4" t="inlineStr">
         <is>
           <t>Спецобъединение РЕФЛЕКТ-2</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+    <row r="37" ht="32" customHeight="1">
+      <c r="A37" s="4" t="inlineStr">
         <is>
           <t>Костюм сигнальный зимний</t>
         </is>
@@ -1093,20 +1102,20 @@
       <c r="B37" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C37" s="4" t="n">
+      <c r="C37" s="5" t="n">
         <v>11621</v>
       </c>
-      <c r="D37" s="4" t="n">
+      <c r="D37" s="5" t="n">
         <v>46484</v>
       </c>
-      <c r="E37" s="2" t="inlineStr">
+      <c r="E37" s="4" t="inlineStr">
         <is>
           <t>Спецобъединение РЕФЛЕКТ-2 зимний</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
+    <row r="38" ht="32" customHeight="1">
+      <c r="A38" s="4" t="inlineStr">
         <is>
           <t>Костюм от нефтепродуктов зимний</t>
         </is>
@@ -1114,20 +1123,20 @@
       <c r="B38" s="2" t="n">
         <v>31</v>
       </c>
-      <c r="C38" s="4" t="n">
+      <c r="C38" s="5" t="n">
         <v>11253</v>
       </c>
-      <c r="D38" s="4" t="n">
+      <c r="D38" s="5" t="n">
         <v>348843</v>
       </c>
-      <c r="E38" s="2" t="inlineStr">
+      <c r="E38" s="4" t="inlineStr">
         <is>
           <t>Тракт ПЛАСТОЙЛ (Спецобъединение 24 199)</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
+    <row r="39" ht="32" customHeight="1">
+      <c r="A39" s="4" t="inlineStr">
         <is>
           <t>Костюм от нефтепродуктов летний</t>
         </is>
@@ -1135,20 +1144,20 @@
       <c r="B39" s="2" t="n">
         <v>56</v>
       </c>
-      <c r="C39" s="4" t="n">
+      <c r="C39" s="5" t="n">
         <v>6731</v>
       </c>
-      <c r="D39" s="4" t="n">
+      <c r="D39" s="5" t="n">
         <v>376936</v>
       </c>
-      <c r="E39" s="2" t="inlineStr">
+      <c r="E39" s="4" t="inlineStr">
         <is>
           <t>Тракт (Спецобъединение 13 219)</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
+    <row r="40" ht="32" customHeight="1">
+      <c r="A40" s="4" t="inlineStr">
         <is>
           <t>Плащ от воды</t>
         </is>
@@ -1156,20 +1165,20 @@
       <c r="B40" s="2" t="n">
         <v>49</v>
       </c>
-      <c r="C40" s="4" t="n">
+      <c r="C40" s="5" t="n">
         <v>971</v>
       </c>
-      <c r="D40" s="4" t="n">
+      <c r="D40" s="5" t="n">
         <v>47579</v>
       </c>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="E40" s="4" t="inlineStr">
         <is>
           <t>Тракт 971 / Фабрикант 1 365</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
+    <row r="41" ht="32" customHeight="1">
+      <c r="A41" s="4" t="inlineStr">
         <is>
           <t>Футболка красная</t>
         </is>
@@ -1177,20 +1186,20 @@
       <c r="B41" s="2" t="n">
         <v>112</v>
       </c>
-      <c r="C41" s="4" t="n">
+      <c r="C41" s="5" t="n">
         <v>300</v>
       </c>
-      <c r="D41" s="4" t="n">
+      <c r="D41" s="5" t="n">
         <v>33600</v>
       </c>
-      <c r="E41" s="2" t="inlineStr">
+      <c r="E41" s="4" t="inlineStr">
         <is>
           <t>Иваново опт 211–270</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
+    <row r="42" ht="32" customHeight="1">
+      <c r="A42" s="4" t="inlineStr">
         <is>
           <t>Халат белый</t>
         </is>
@@ -1198,20 +1207,20 @@
       <c r="B42" s="2" t="n">
         <v>70</v>
       </c>
-      <c r="C42" s="4" t="n">
+      <c r="C42" s="5" t="n">
         <v>735</v>
       </c>
-      <c r="D42" s="4" t="n">
+      <c r="D42" s="5" t="n">
         <v>51450</v>
       </c>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="E42" s="4" t="inlineStr">
         <is>
           <t>ivuniforma 721–770</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr">
+    <row r="43" ht="32" customHeight="1">
+      <c r="A43" s="4" t="inlineStr">
         <is>
           <t>Халат синий</t>
         </is>
@@ -1219,115 +1228,116 @@
       <c r="B43" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="C43" s="4" t="n">
+      <c r="C43" s="5" t="n">
         <v>735</v>
       </c>
-      <c r="D43" s="4" t="n">
+      <c r="D43" s="5" t="n">
         <v>7350</v>
       </c>
-      <c r="E43" s="2" t="inlineStr">
+      <c r="E43" s="4" t="inlineStr">
         <is>
           <t>ivuniforma 735</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="5" t="inlineStr">
+    <row r="44" ht="32" customHeight="1">
+      <c r="A44" s="6" t="inlineStr">
         <is>
           <t>Закупка итого</t>
         </is>
       </c>
       <c r="B44" s="2" t="n"/>
       <c r="C44" s="2" t="n"/>
-      <c r="D44" s="6" t="n">
+      <c r="D44" s="7" t="n">
         <v>1132385</v>
       </c>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="E44" s="4" t="inlineStr">
         <is>
           <t>Цен за ед. в ЕИС нет — НМЦК 3,64 млн против нашей закупки; проверить ТЗ (ткани/логотипы)</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
+    <row r="45" ht="32" customHeight="1">
+      <c r="A45" s="6" t="inlineStr">
         <is>
           <t>Доставка</t>
         </is>
       </c>
       <c r="B45" s="2" t="n"/>
       <c r="C45" s="2" t="n"/>
-      <c r="D45" s="6" t="n">
+      <c r="D45" s="7" t="n">
         <v>38303</v>
       </c>
       <c r="E45" s="2" t="n"/>
     </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr">
+    <row r="46" ht="32" customHeight="1">
+      <c r="A46" s="6" t="inlineStr">
         <is>
           <t>НМЦК</t>
         </is>
       </c>
       <c r="B46" s="2" t="n"/>
       <c r="C46" s="2" t="n"/>
-      <c r="D46" s="6" t="n">
+      <c r="D46" s="7" t="n">
         <v>3637476.36</v>
       </c>
       <c r="E46" s="2" t="n"/>
     </row>
-    <row r="47">
-      <c r="A47" s="5" t="inlineStr">
+    <row r="47" ht="32" customHeight="1">
+      <c r="A47" s="6" t="inlineStr">
         <is>
           <t>Маржа при НМЦК</t>
         </is>
       </c>
       <c r="B47" s="2" t="n"/>
       <c r="C47" s="2" t="n"/>
-      <c r="D47" s="7" t="n">
+      <c r="D47" s="8" t="n">
         <v>0.6781592829375803</v>
       </c>
       <c r="E47" s="2" t="n"/>
     </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr">
+    <row r="48" ht="32" customHeight="1">
+      <c r="A48" s="6" t="inlineStr">
         <is>
           <t>Чистая прибыль при НМЦК</t>
         </is>
       </c>
       <c r="B48" s="2" t="n"/>
       <c r="C48" s="2" t="n"/>
-      <c r="D48" s="6" t="n">
+      <c r="D48" s="7" t="n">
         <v>2039320.150039671</v>
       </c>
       <c r="E48" s="2" t="n"/>
     </row>
-    <row r="49">
-      <c r="A49" s="5" t="inlineStr">
+    <row r="49" ht="32" customHeight="1">
+      <c r="A49" s="6" t="inlineStr">
         <is>
           <t>Чистая прибыль при снижении 10%</t>
         </is>
       </c>
       <c r="B49" s="2" t="n"/>
       <c r="C49" s="2" t="n"/>
-      <c r="D49" s="6" t="n">
+      <c r="D49" s="7" t="n">
         <v>1732608.143364471</v>
       </c>
       <c r="E49" s="2" t="n"/>
     </row>
-    <row r="50">
-      <c r="A50" s="5" t="inlineStr">
+    <row r="50" ht="32" customHeight="1">
+      <c r="A50" s="6" t="inlineStr">
         <is>
           <t>Безубыток до снижения</t>
         </is>
       </c>
       <c r="B50" s="2" t="n"/>
       <c r="C50" s="2" t="n"/>
-      <c r="D50" s="7" t="n">
+      <c r="D50" s="8" t="n">
         <v>0.6648973974466078</v>
       </c>
       <c r="E50" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -1335,7 +1345,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:H33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -1350,1259 +1360,1259 @@
     <col width="60" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+    <row r="1" ht="48" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Группа товара</t>
         </is>
       </c>
-      <c r="B1" s="8" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Сайт</t>
         </is>
       </c>
-      <c r="C1" s="8" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Производитель / город</t>
         </is>
       </c>
-      <c r="D1" s="8" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Модели</t>
         </is>
       </c>
-      <c r="E1" s="8" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Цена от, ₽</t>
         </is>
       </c>
-      <c r="F1" s="8" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Цена до, ₽</t>
         </is>
       </c>
-      <c r="G1" s="8" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Тип цены</t>
         </is>
       </c>
-      <c r="H1" s="8" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Ссылка</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>Летний рабочий костюм</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>ivuniforma.ru</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>Иваново, фабрика</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>Р-02-3-ГР / Р-02-21-ГР / Р-02-184-ГР</t>
         </is>
       </c>
-      <c r="E2" s="9" t="n">
+      <c r="E2" s="5" t="n">
         <v>938</v>
       </c>
-      <c r="F2" s="9" t="n">
+      <c r="F2" s="5" t="n">
         <v>1715</v>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>опт</t>
         </is>
       </c>
-      <c r="H2" s="10" t="inlineStr">
+      <c r="H2" s="11" t="inlineStr">
         <is>
           <t>https://www.ivuniforma.ru/catalog/rabochaya-odezhda/letnyaya-spetsodezhda/kostumy/</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="3" ht="32" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>Летний рабочий костюм</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>spets.ru</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>ГК Спецобъединение (Москва)</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>ОПЕРАТОР / СТРОЙМАСТЕР / ДЮРАБЛ</t>
         </is>
       </c>
-      <c r="E3" s="9" t="n">
+      <c r="E3" s="5" t="n">
         <v>3367</v>
       </c>
-      <c r="F3" s="9" t="n">
+      <c r="F3" s="5" t="n">
         <v>4984</v>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="4" t="inlineStr">
         <is>
           <t>прайс с НДС</t>
         </is>
       </c>
-      <c r="H3" s="10" t="inlineStr">
+      <c r="H3" s="11" t="inlineStr">
         <is>
           <t>https://www.spets.ru/products/spetsodezhda/letnyaya/</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Летний рабочий костюм</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>trakt.ru</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Тракт (Москва)</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>РИТМ / ШКВАЛ / МАСТАК</t>
         </is>
       </c>
-      <c r="E4" s="9" t="n">
+      <c r="E4" s="5" t="n">
         <v>3086</v>
       </c>
-      <c r="F4" s="9" t="n">
+      <c r="F4" s="5" t="n">
         <v>3746</v>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>прайс для юрлиц с НДС</t>
         </is>
       </c>
-      <c r="H4" s="10" t="inlineStr">
+      <c r="H4" s="11" t="inlineStr">
         <is>
           <t>https://www.trakt.ru/product/11954/</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Летний костюм МЧС/спасателя</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>voen36.ru</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Воен36 (Воронеж, собств. пр-во)</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>габардин / рип-стоп / ПЭВ</t>
         </is>
       </c>
-      <c r="E5" s="9" t="n">
+      <c r="E5" s="5" t="n">
         <v>3100</v>
       </c>
-      <c r="F5" s="9" t="n">
+      <c r="F5" s="5" t="n">
         <v>5995</v>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>розница</t>
         </is>
       </c>
-      <c r="H5" s="10" t="inlineStr">
+      <c r="H5" s="11" t="inlineStr">
         <is>
           <t>https://voen36.ru/catalog/forma_mchs/</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Летний костюм МЧС/спасателя</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>barrakuda.biz</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>Барракуда (Москва)</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>рип-стоп / п/в</t>
         </is>
       </c>
-      <c r="E6" s="9" t="n">
+      <c r="E6" s="5" t="n">
         <v>4900</v>
       </c>
-      <c r="F6" s="9" t="n">
+      <c r="F6" s="5" t="n">
         <v>6675</v>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>розница, есть опт</t>
         </is>
       </c>
-      <c r="H6" s="10" t="inlineStr">
+      <c r="H6" s="11" t="inlineStr">
         <is>
           <t>https://barrakuda.biz/formennaya-odezhda/kostyumy-mchs</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="7" ht="32" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Летний костюм МЧС/спасателя</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>productcenter.ru</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>«Аврора» (Барнаул, фабрика)</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>полевой МЧС</t>
         </is>
       </c>
-      <c r="E7" s="9" t="n">
+      <c r="E7" s="5" t="n">
         <v>2490</v>
       </c>
-      <c r="F7" s="9" t="n">
+      <c r="F7" s="5" t="n">
         <v>2490</v>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>опт «от»</t>
         </is>
       </c>
-      <c r="H7" s="10" t="inlineStr">
+      <c r="H7" s="11" t="inlineStr">
         <is>
           <t>https://productcenter.ru/products/45461/kostiumy-dlia-sotrudnikov-mchs</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+    <row r="8" ht="32" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Летний полевой костюм</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>ivsoteks.ru</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>Ивсотекс (Иваново)</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>Святогор Greta / Горка Rip-stop</t>
         </is>
       </c>
-      <c r="E8" s="9" t="n">
+      <c r="E8" s="5" t="n">
         <v>1600</v>
       </c>
-      <c r="F8" s="9" t="n">
+      <c r="F8" s="5" t="n">
         <v>2490</v>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>опт</t>
         </is>
       </c>
-      <c r="H8" s="10" t="inlineStr">
+      <c r="H8" s="11" t="inlineStr">
         <is>
           <t>https://ivsoteks.ru/specodejda</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="9" ht="32" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Летний полевой костюм</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>splav.ru</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Сплав (СПб, фабрика)</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>Костюм полевой Сплав</t>
         </is>
       </c>
-      <c r="E9" s="9" t="n">
+      <c r="E9" s="5" t="n">
         <v>4600</v>
       </c>
-      <c r="F9" s="9" t="n">
+      <c r="F9" s="5" t="n">
         <v>8700</v>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>розница</t>
         </is>
       </c>
-      <c r="H9" s="10" t="inlineStr">
+      <c r="H9" s="11" t="inlineStr">
         <is>
           <t>https://www.splav.ru/catalog/military-tactics/novyj-odezhda/kostyumy/letnie-kostyumy/</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Зимний рабочий костюм</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>ivuniforma.ru</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>Иваново, фабрика</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>Р-02-66 / Р-02-45 / Р-02-61</t>
         </is>
       </c>
-      <c r="E10" s="9" t="n">
+      <c r="E10" s="5" t="n">
         <v>3549</v>
       </c>
-      <c r="F10" s="9" t="n">
+      <c r="F10" s="5" t="n">
         <v>5810</v>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>опт</t>
         </is>
       </c>
-      <c r="H10" s="10" t="inlineStr">
+      <c r="H10" s="11" t="inlineStr">
         <is>
           <t>https://www.ivuniforma.ru/catalog/rabochaya-odezhda/zimnjaja/kostyumy-1/</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Зимний рабочий костюм</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>specteks37.ru</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>СпецТекс 37 (Иваново)</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>№1 / №2 / №265 (IV пояс)</t>
         </is>
       </c>
-      <c r="E11" s="9" t="n">
+      <c r="E11" s="5" t="n">
         <v>2650</v>
       </c>
-      <c r="F11" s="9" t="n">
+      <c r="F11" s="5" t="n">
         <v>4600</v>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G11" s="4" t="inlineStr">
         <is>
           <t>опт «от»</t>
         </is>
       </c>
-      <c r="H11" s="10" t="inlineStr">
+      <c r="H11" s="11" t="inlineStr">
         <is>
           <t>https://www.specteks37.ru/katalog/zimnyaya-spetsodezhda/</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="12" ht="32" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Зимний рабочий костюм</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>spec-standart.ru</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>Стандарт Спецодежда (Иваново)</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>Сибирь / Зимний / Север (тройка)</t>
         </is>
       </c>
-      <c r="E12" s="9" t="n">
+      <c r="E12" s="5" t="n">
         <v>4158</v>
       </c>
-      <c r="F12" s="9" t="n">
+      <c r="F12" s="5" t="n">
         <v>8543</v>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr">
         <is>
           <t>«от»</t>
         </is>
       </c>
-      <c r="H12" s="10" t="inlineStr">
+      <c r="H12" s="11" t="inlineStr">
         <is>
           <t>https://spec-standart.ru/zimnyaya-specodezhda</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Зимний рабочий костюм</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>ivsoteks.ru</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Ивсотекс (Иваново)</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>Святогор / Урал / Привал</t>
         </is>
       </c>
-      <c r="E13" s="9" t="n">
+      <c r="E13" s="5" t="n">
         <v>3520</v>
       </c>
-      <c r="F13" s="9" t="n">
+      <c r="F13" s="5" t="n">
         <v>5830</v>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="G13" s="4" t="inlineStr">
         <is>
           <t>опт</t>
         </is>
       </c>
-      <c r="H13" s="10" t="inlineStr">
+      <c r="H13" s="11" t="inlineStr">
         <is>
           <t>https://ivsoteks.ru/specodejda</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+    <row r="14" ht="32" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Зимний рабочий костюм</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>spets.ru</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>ГК Спецобъединение</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>УРЕНГОЙ / СИБИРЬ / НАДЫМ / УРАГАН</t>
         </is>
       </c>
-      <c r="E14" s="9" t="n">
+      <c r="E14" s="5" t="n">
         <v>6084</v>
       </c>
-      <c r="F14" s="9" t="n">
+      <c r="F14" s="5" t="n">
         <v>15250</v>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>прайс с НДС</t>
         </is>
       </c>
-      <c r="H14" s="10" t="inlineStr">
+      <c r="H14" s="11" t="inlineStr">
         <is>
           <t>https://www.spets.ru/products/spetsodezhda/odezhda_zimnyaya/</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>Зимний рабочий костюм</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>trakt.ru</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>Тракт</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>ВАХТА / ДЖОБЕР / БРИГАДИР / ФРОСТ</t>
         </is>
       </c>
-      <c r="E15" s="9" t="n">
+      <c r="E15" s="5" t="n">
         <v>3588</v>
       </c>
-      <c r="F15" s="9" t="n">
+      <c r="F15" s="5" t="n">
         <v>7793</v>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>прайс для юрлиц с НДС</t>
         </is>
       </c>
-      <c r="H15" s="10" t="inlineStr">
+      <c r="H15" s="11" t="inlineStr">
         <is>
           <t>https://www.trakt.ru/product/12066/</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    <row r="16" ht="32" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Зимний костюм северный (IV/особый пояс)</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>spets.ru</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>ГК Спецобъединение</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>НАДЫМ / УРАГАН-УЛЬТРА</t>
         </is>
       </c>
-      <c r="E16" s="9" t="n">
+      <c r="E16" s="5" t="n">
         <v>9760</v>
       </c>
-      <c r="F16" s="9" t="n">
+      <c r="F16" s="5" t="n">
         <v>22875</v>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="G16" s="4" t="inlineStr">
         <is>
           <t>прайс с НДС</t>
         </is>
       </c>
-      <c r="H16" s="10" t="inlineStr">
+      <c r="H16" s="11" t="inlineStr">
         <is>
           <t>https://www.spets.ru/products/spetsodezhda/odezhda_zimnyaya/</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+    <row r="17" ht="32" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>Зимний костюм северный (IV/особый пояс)</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>trakt.ru</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>Тракт</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>БЕРИНГ / СЕВЕРНЫЙ ШЕЛЬФ (куртка+п/к)</t>
         </is>
       </c>
-      <c r="E17" s="9" t="n">
+      <c r="E17" s="5" t="n">
         <v>9659</v>
       </c>
-      <c r="F17" s="9" t="n">
+      <c r="F17" s="5" t="n">
         <v>23998</v>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="G17" s="4" t="inlineStr">
         <is>
           <t>прайс для юрлиц с НДС</t>
         </is>
       </c>
-      <c r="H17" s="10" t="inlineStr">
+      <c r="H17" s="11" t="inlineStr">
         <is>
           <t>https://www.trakt.ru/product/13086/</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
+    <row r="18" ht="32" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Зимний костюм спасателя МЧС</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>barrakuda.biz</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>Барракуда</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>поливискоза, с капюшоном</t>
         </is>
       </c>
-      <c r="E18" s="9" t="n">
+      <c r="E18" s="5" t="n">
         <v>14461</v>
       </c>
-      <c r="F18" s="9" t="n">
+      <c r="F18" s="5" t="n">
         <v>14461</v>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="G18" s="4" t="inlineStr">
         <is>
           <t>розница</t>
         </is>
       </c>
-      <c r="H18" s="10" t="inlineStr">
+      <c r="H18" s="11" t="inlineStr">
         <is>
           <t>https://barrakuda.biz/formennaya-odezhda/kostyumy-mchs</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
+    <row r="19" ht="32" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Зимняя куртка МЧС</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>voen36.ru</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>Воен36</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>уставная / удлинённая</t>
         </is>
       </c>
-      <c r="E19" s="9" t="n">
+      <c r="E19" s="5" t="n">
         <v>4800</v>
       </c>
-      <c r="F19" s="9" t="n">
+      <c r="F19" s="5" t="n">
         <v>7150</v>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="G19" s="4" t="inlineStr">
         <is>
           <t>розница</t>
         </is>
       </c>
-      <c r="H19" s="10" t="inlineStr">
+      <c r="H19" s="11" t="inlineStr">
         <is>
           <t>https://voen36.ru/catalog/forma_mchs/</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
+    <row r="20" ht="32" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Комбинезон летний</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>ivuniforma.ru</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>Иваново, фабрика</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>Р-11-87 / Р-11-88</t>
         </is>
       </c>
-      <c r="E20" s="9" t="n">
+      <c r="E20" s="5" t="n">
         <v>3766</v>
       </c>
-      <c r="F20" s="9" t="n">
+      <c r="F20" s="5" t="n">
         <v>4102</v>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="G20" s="4" t="inlineStr">
         <is>
           <t>опт</t>
         </is>
       </c>
-      <c r="H20" s="10" t="inlineStr">
+      <c r="H20" s="11" t="inlineStr">
         <is>
           <t>https://www.ivuniforma.ru/catalog/rabochaya-odezhda/letnyaya-spetsodezhda/kombinezony/</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
+    <row r="21" ht="32" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Комбинезон зимний</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>spets.ru</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>ГК Спецобъединение</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr">
         <is>
           <t>ПИЛОТ зимний</t>
         </is>
       </c>
-      <c r="E21" s="9" t="n">
+      <c r="E21" s="5" t="n">
         <v>10199</v>
       </c>
-      <c r="F21" s="9" t="n">
+      <c r="F21" s="5" t="n">
         <v>10577</v>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="G21" s="4" t="inlineStr">
         <is>
           <t>прайс с НДС</t>
         </is>
       </c>
-      <c r="H21" s="10" t="inlineStr">
+      <c r="H21" s="11" t="inlineStr">
         <is>
           <t>https://www.spets.ru/products/spetsodezhda/odezhda_zimnyaya/</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
+    <row r="22" ht="32" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Футболка</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>spets.ru</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>ГК Спецобъединение</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t>160 г/м², кор. рукав</t>
         </is>
       </c>
-      <c r="E22" s="9" t="n">
+      <c r="E22" s="5" t="n">
         <v>488</v>
       </c>
-      <c r="F22" s="9" t="n">
+      <c r="F22" s="5" t="n">
         <v>488</v>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="G22" s="4" t="inlineStr">
         <is>
           <t>прайс с НДС</t>
         </is>
       </c>
-      <c r="H22" s="10" t="inlineStr">
+      <c r="H22" s="11" t="inlineStr">
         <is>
           <t>https://www.spets.ru/products/spetsodezhda/trikotazh/</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
+    <row r="23" ht="32" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>Футболка</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>trakt.ru</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>Тракт</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr">
         <is>
           <t>Футболка синяя</t>
         </is>
       </c>
-      <c r="E23" s="9" t="n">
+      <c r="E23" s="5" t="n">
         <v>484</v>
       </c>
-      <c r="F23" s="9" t="n">
+      <c r="F23" s="5" t="n">
         <v>484</v>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="G23" s="4" t="inlineStr">
         <is>
           <t>прайс</t>
         </is>
       </c>
-      <c r="H23" s="10" t="inlineStr">
+      <c r="H23" s="11" t="inlineStr">
         <is>
           <t>https://www.trakt.ru/product/12012/</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
+    <row r="24" ht="32" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Футболка</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>productcenter.ru</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>фабрики Иваново</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t>мужская футболка</t>
         </is>
       </c>
-      <c r="E24" s="9" t="n">
+      <c r="E24" s="5" t="n">
         <v>211</v>
       </c>
-      <c r="F24" s="9" t="n">
+      <c r="F24" s="5" t="n">
         <v>270</v>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="G24" s="4" t="inlineStr">
         <is>
           <t>опт «от»</t>
         </is>
       </c>
-      <c r="H24" s="10" t="inlineStr">
+      <c r="H24" s="11" t="inlineStr">
         <is>
           <t>https://productcenter.ru/products/r-ivanovskaia-obl-168/c-ivanovo-2550/catalog-muzhskiie-futbolki-1062</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
+    <row r="25" ht="32" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>Халат рабочий</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>ivuniforma.ru</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="4" t="inlineStr">
         <is>
           <t>Иваново, фабрика</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="4" t="inlineStr">
         <is>
           <t>Р-20-104 / Р-20-251 / Р-20-256</t>
         </is>
       </c>
-      <c r="E25" s="9" t="n">
+      <c r="E25" s="5" t="n">
         <v>609</v>
       </c>
-      <c r="F25" s="9" t="n">
+      <c r="F25" s="5" t="n">
         <v>1064</v>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="G25" s="4" t="inlineStr">
         <is>
           <t>опт</t>
         </is>
       </c>
-      <c r="H25" s="10" t="inlineStr">
+      <c r="H25" s="11" t="inlineStr">
         <is>
           <t>https://www.ivuniforma.ru/catalog/rabochaya-odezhda/letnyaya-spetsodezhda/khalati/</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
+    <row r="26" ht="32" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>Халат рабочий</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>fabrikant-textile.ru</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>Фабрикант (Иваново)</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr">
         <is>
           <t>халат женский смесовка</t>
         </is>
       </c>
-      <c r="E26" s="9" t="n">
+      <c r="E26" s="5" t="n">
         <v>400</v>
       </c>
-      <c r="F26" s="9" t="n">
+      <c r="F26" s="5" t="n">
         <v>400</v>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="G26" s="4" t="inlineStr">
         <is>
           <t>«от»</t>
         </is>
       </c>
-      <c r="H26" s="10" t="inlineStr">
+      <c r="H26" s="11" t="inlineStr">
         <is>
           <t>https://fabrikant-textile.ru/catalog/spetsodezhda/</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
+    <row r="27" ht="32" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t>Жилет утепленный</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>ivuniforma.ru</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>Иваново, фабрика</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="4" t="inlineStr">
         <is>
           <t>Р-06-112 / Р-06-206</t>
         </is>
       </c>
-      <c r="E27" s="9" t="n">
+      <c r="E27" s="5" t="n">
         <v>1190</v>
       </c>
-      <c r="F27" s="9" t="n">
+      <c r="F27" s="5" t="n">
         <v>1372</v>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="G27" s="4" t="inlineStr">
         <is>
           <t>опт</t>
         </is>
       </c>
-      <c r="H27" s="10" t="inlineStr">
+      <c r="H27" s="11" t="inlineStr">
         <is>
           <t>https://www.ivuniforma.ru/catalog/rabochaya-odezhda/zimnjaja/</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
+    <row r="28" ht="32" customHeight="1">
+      <c r="A28" s="4" t="inlineStr">
         <is>
           <t>Жилет утепленный</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>spets.ru</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>ГК Спецобъединение</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="4" t="inlineStr">
         <is>
           <t>САТУРН</t>
         </is>
       </c>
-      <c r="E28" s="9" t="n">
+      <c r="E28" s="5" t="n">
         <v>2788</v>
       </c>
-      <c r="F28" s="9" t="n">
+      <c r="F28" s="5" t="n">
         <v>2788</v>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="G28" s="4" t="inlineStr">
         <is>
           <t>прайс с НДС</t>
         </is>
       </c>
-      <c r="H28" s="10" t="inlineStr">
+      <c r="H28" s="11" t="inlineStr">
         <is>
           <t>https://www.spets.ru/products/spetsodezhda/odezhda_dlya_okhrannykh_struktur/</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
+    <row r="29" ht="32" customHeight="1">
+      <c r="A29" s="4" t="inlineStr">
         <is>
           <t>Жилет сигнальный</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>spets.ru</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>ГК Спецобъединение</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="4" t="inlineStr">
         <is>
           <t>сигнальный / ГОСТ</t>
         </is>
       </c>
-      <c r="E29" s="9" t="n">
+      <c r="E29" s="5" t="n">
         <v>390</v>
       </c>
-      <c r="F29" s="9" t="n">
+      <c r="F29" s="5" t="n">
         <v>677</v>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="G29" s="4" t="inlineStr">
         <is>
           <t>прайс с НДС</t>
         </is>
       </c>
-      <c r="H29" s="10" t="inlineStr">
+      <c r="H29" s="11" t="inlineStr">
         <is>
           <t>https://www.spets.ru/products/spetsodezhda/odezhda_spetsialnaya/</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
+    <row r="30" ht="32" customHeight="1">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>Жилет сигнальный</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <t>fabrikant-textile.ru</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="4" t="inlineStr">
         <is>
           <t>Фабрикант (Иваново)</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" s="4" t="inlineStr">
         <is>
           <t>с СОП</t>
         </is>
       </c>
-      <c r="E30" s="9" t="n">
+      <c r="E30" s="5" t="n">
         <v>260</v>
       </c>
-      <c r="F30" s="9" t="n">
+      <c r="F30" s="5" t="n">
         <v>320</v>
       </c>
-      <c r="G30" t="inlineStr">
+      <c r="G30" s="4" t="inlineStr">
         <is>
           <t>«от»</t>
         </is>
       </c>
-      <c r="H30" s="10" t="inlineStr">
+      <c r="H30" s="11" t="inlineStr">
         <is>
           <t>https://fabrikant-textile.ru/catalog/spetsodezhda/</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
+    <row r="31" ht="32" customHeight="1">
+      <c r="A31" s="4" t="inlineStr">
         <is>
           <t>Костюм от нефтепродуктов</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>spets.ru</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="4" t="inlineStr">
         <is>
           <t>ГК Спецобъединение</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="4" t="inlineStr">
         <is>
           <t>МЕГАСТАТОЙЛ летний / зимний</t>
         </is>
       </c>
-      <c r="E31" s="9" t="n">
+      <c r="E31" s="5" t="n">
         <v>13219</v>
       </c>
-      <c r="F31" s="9" t="n">
+      <c r="F31" s="5" t="n">
         <v>24199</v>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="G31" s="4" t="inlineStr">
         <is>
           <t>прайс с НДС</t>
         </is>
       </c>
-      <c r="H31" s="10" t="inlineStr">
+      <c r="H31" s="11" t="inlineStr">
         <is>
           <t>https://www.spets.ru/products/spetsodezhda/odezhda_spetsialnaya/</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
+    <row r="32" ht="32" customHeight="1">
+      <c r="A32" s="4" t="inlineStr">
         <is>
           <t>Костюм от нефтепродуктов</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t>trakt.ru</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="4" t="inlineStr">
         <is>
           <t>Тракт</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" s="4" t="inlineStr">
         <is>
           <t>летний 12492 / ПЛАСТОЙЛ зимний</t>
         </is>
       </c>
-      <c r="E32" s="9" t="n">
+      <c r="E32" s="5" t="n">
         <v>6731</v>
       </c>
-      <c r="F32" s="9" t="n">
+      <c r="F32" s="5" t="n">
         <v>11253</v>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="G32" s="4" t="inlineStr">
         <is>
           <t>прайс для юрлиц с НДС</t>
         </is>
       </c>
-      <c r="H32" s="10" t="inlineStr">
+      <c r="H32" s="11" t="inlineStr">
         <is>
           <t>https://www.trakt.ru/product/12720/</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
+    <row r="33" ht="32" customHeight="1">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>Костюм сигнальный</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>spets.ru</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="4" t="inlineStr">
         <is>
           <t>ГК Спецобъединение</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" s="4" t="inlineStr">
         <is>
           <t>РЕФЛЕКТ-1/2 летний / зимний</t>
         </is>
       </c>
-      <c r="E33" s="9" t="n">
+      <c r="E33" s="5" t="n">
         <v>6112</v>
       </c>
-      <c r="F33" s="9" t="n">
+      <c r="F33" s="5" t="n">
         <v>12780</v>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="G33" s="4" t="inlineStr">
         <is>
           <t>прайс с НДС</t>
         </is>
       </c>
-      <c r="H33" s="10" t="inlineStr">
+      <c r="H33" s="11" t="inlineStr">
         <is>
           <t>https://www.spets.ru/products/spetsodezhda/odezhda_spetsialnaya/</t>
         </is>
@@ -2645,5 +2655,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId32"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>